<commit_message>
Claude: figuras y código de figuras (3.B.35)
</commit_message>
<xml_diff>
--- a/Ejercicio-3/Parte-B/3.B.35/Code/datos/tablas_figuras.xlsx
+++ b/Ejercicio-3/Parte-B/3.B.35/Code/datos/tablas_figuras.xlsx
@@ -49,6 +49,7 @@
     <sheet name="MCCA_complementariedad" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="MCCA_saldos" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="MCCA_reparto_manuf" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="MERCOSUR_tipo_cambio" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37884,6 +37885,543 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tipo de cambio real bilateral peso argentino-real (índice 1995 = 100) y saldo comercial de Argentina con Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Banco Mundial (WDI): tipos de cambio oficiales (PA.NUS.FCRF) y deflactores del PIB (NY.GDP.DEFL.ZS), porque WDI no tiene el IPC argentino; saldo con las exportaciones declaradas por cada país (Code/datos_comercio.py). Cálculo propio (Code/figuras_afinidad.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tipo de cambio real (1995 = 100)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Saldo de Argentina con Brasil (miles de millones USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1980</v>
+      </c>
+      <c r="B5" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.33</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B6" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.29</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1982</v>
+      </c>
+      <c r="B7" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1983</v>
+      </c>
+      <c r="B8" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B9" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-0.37</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1985</v>
+      </c>
+      <c r="B10" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1986</v>
+      </c>
+      <c r="B11" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B12" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1988</v>
+      </c>
+      <c r="B13" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1989</v>
+      </c>
+      <c r="B14" t="n">
+        <v>132.2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1990</v>
+      </c>
+      <c r="B15" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1991</v>
+      </c>
+      <c r="B16" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1992</v>
+      </c>
+      <c r="B17" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-1.37</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1993</v>
+      </c>
+      <c r="B18" t="n">
+        <v>56</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-0.84</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B19" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B20" t="n">
+        <v>100</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B21" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B22" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B23" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B24" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B25" t="n">
+        <v>79</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B26" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B27" t="n">
+        <v>139.5</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B28" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B29" t="n">
+        <v>125</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-1.96</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B30" t="n">
+        <v>145.2</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-3.64</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B31" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-3.59</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B32" t="n">
+        <v>168.3</v>
+      </c>
+      <c r="C32" t="n">
+        <v>-3.92</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B33" t="n">
+        <v>160.3</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-4.33</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B34" t="n">
+        <v>161.3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B35" t="n">
+        <v>172.7</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-4.07</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B36" t="n">
+        <v>167.7</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-5.38</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B37" t="n">
+        <v>140</v>
+      </c>
+      <c r="C37" t="n">
+        <v>-1.53</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B38" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-3.66</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B39" t="n">
+        <v>137.9</v>
+      </c>
+      <c r="C39" t="n">
+        <v>-0.39</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B40" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-2.7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B41" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="C41" t="n">
+        <v>-4.38</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B42" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="C42" t="n">
+        <v>-8.31</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B43" t="n">
+        <v>121.7</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-3.62</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B44" t="n">
+        <v>135</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B45" t="n">
+        <v>115</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B46" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B47" t="n">
+        <v>100.4</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-2.71</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B48" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-4.86</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B49" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Marcelo: cambios propios, guardados antes de una acción de Claude (3.B.35)
</commit_message>
<xml_diff>
--- a/Ejercicio-3/Parte-B/3.B.35/Code/datos/tablas_figuras.xlsx
+++ b/Ejercicio-3/Parte-B/3.B.35/Code/datos/tablas_figuras.xlsx
@@ -57,11 +57,11 @@
     <sheet name="MERCOSUR_reparto_manuf" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="CEFTA_convergencia" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="CEFTA_ancla" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="AFCFTA_composicion" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="AFCFTA_materias" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="AFCFTA_aranceles" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="PAFTA_sin_petroleo" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="PAFTA_composicion" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="AFCFTA_materias" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="AFCFTA_aranceles" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="PAFTA_sin_petroleo" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="PAFTA_composicion" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="AFCFTA_composicion" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51087,237 +51087,371 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Manufacturas en las exportaciones de los países africanos a África y fuera de África (%)</t>
+          <t>Estructura de las exportaciones de las grandes economías africanas y complementariedad entre ellas, 2023</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WITS (Banco Mundial), grupo «manuf» (CUCI 5 a 8 sin 667 y 68) y total, exportaciones declaradas por cada país a cada socio; solo los países que declaran cada año. Cálculo propio (Code/figuras_afinidad.py).</t>
+          <t>WITS (Banco Mundial): exportaciones por grupos de la CUCI (alimentos, materias primas agrícolas, combustibles, minerales y metales, manufacturas) y exportaciones e importaciones por las 16 secciones del SA de WITS (complementariedad aproximada, MICHAELY, 1996). Cálculo propio (Code/figuras_afinidad.py).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Año</t>
+          <t>País</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A África (%)</t>
+          <t>Alimentos (%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fuera de África (%)</t>
+          <t>Materias primas agrícolas (%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Países que declaran</t>
+          <t>Combustibles (%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AGO 2023: África / fuera</t>
+          <t>Minerales y metales (%)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TUN 2023: África / fuera</t>
+          <t>Manufacturas (%)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MAR 2023: África / fuera</t>
+          <t>Otros (%)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EGY 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ZAF 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>KEN 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>GHA 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>CIV 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>TZA 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>ETH 2023: África / fuera</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>NGA 2023: África / fuera</t>
+          <t>Complementariedad media con los demás</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>2000</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TUN</t>
+        </is>
       </c>
       <c r="B5" t="n">
-        <v>40.6</v>
+        <v>12.8</v>
       </c>
       <c r="C5" t="n">
-        <v>26.2</v>
+        <v>0.3</v>
       </c>
       <c r="D5" t="n">
-        <v>39</v>
+        <v>6.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>63.5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>2005</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
       </c>
       <c r="B6" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>61.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EGY</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F7" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>67.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ZAF</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>61.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>45.3</v>
       </c>
-      <c r="C6" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B7" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="C7" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B8" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="C8" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="D8" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B9" t="n">
-        <v>49.3</v>
-      </c>
       <c r="C9" t="n">
-        <v>24.5</v>
+        <v>11.3</v>
       </c>
       <c r="D9" t="n">
-        <v>43</v>
+        <v>5.2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>47.9</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>2023</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CIV</t>
+        </is>
       </c>
       <c r="B10" t="n">
-        <v>48.8</v>
+        <v>44.3</v>
       </c>
       <c r="C10" t="n">
-        <v>26.5</v>
+        <v>12.4</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>72.8 / 2.4</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>71.9 / 80.0</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>70.9 / 75.2</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>69.0 / 48.2</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>61.9 / 32.9</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>57.6 / 14.3</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>33.3 / 1.2</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>32.7 / 6.8</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>27.4 / 5.3</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>13.9 / 8.4</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>8.5 / 2.2</t>
-        </is>
+        <v>15.8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>48.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TZA</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F11" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GHA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>18</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NGA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>29.7</v>
       </c>
     </row>
   </sheetData>
@@ -51331,20 +51465,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Estructura de las exportaciones de las grandes economías africanas y complementariedad entre ellas, 2023</t>
+          <t>Arancel aplicado y de nación más favorecida de los países africanos según el origen de las importaciones (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WITS (Banco Mundial): exportaciones por grupos de la CUCI (alimentos, materias primas agrícolas, combustibles, minerales y metales, manufacturas) y exportaciones e importaciones por las 16 secciones del SA de WITS (complementariedad aproximada, MICHAELY, 1996). Cálculo propio (Code/figuras_afinidad.py).</t>
+          <t>WITS (Banco Mundial), tradestats-tariff: AHS-WGHTD-AVRG y MFN-WGHTD-AVRG por socio, ponderados por las importaciones de cada socio (MPRT-TRD-VL); último año disponible entre 2019 y 2022. Comunidad = socio de la misma comunidad con libre comercio (CEDEAO, CEEAC, EAC, COMESA, SADC, UEMOA, CEMAC). Cálculo propio (Code/figuras_afinidad.py).</t>
         </is>
       </c>
     </row>
@@ -51356,346 +51490,1043 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alimentos (%)</t>
+          <t>Año</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Materias primas agrícolas (%)</t>
+          <t>Aplicado, comunidad</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Combustibles (%)</t>
+          <t>Aplicado, resto de África</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Minerales y metales (%)</t>
+          <t>Aplicado, fuera de África</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Manufacturas (%)</t>
+          <t>NMF, a África</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Otros (%)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Complementariedad media con los demás</t>
+          <t>Importaciones desde África (USD)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TUN</t>
+          <t>AGO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.8</v>
+        <v>2021</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3</v>
+        <v>19.71</v>
       </c>
       <c r="D5" t="n">
-        <v>6.2</v>
+        <v>13.39</v>
       </c>
       <c r="E5" t="n">
-        <v>1.3</v>
+        <v>12.07</v>
       </c>
       <c r="F5" t="n">
-        <v>79.2</v>
+        <v>15.64</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>63.5</v>
+        <v>1204584255.78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>BDI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.8</v>
+        <v>2021</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6</v>
+        <v>0.14</v>
       </c>
       <c r="D6" t="n">
-        <v>1.2</v>
+        <v>15.96</v>
       </c>
       <c r="E6" t="n">
-        <v>4.4</v>
+        <v>9.17</v>
       </c>
       <c r="F6" t="n">
-        <v>74.90000000000001</v>
+        <v>24.36</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>61.9</v>
+        <v>308315205.21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EGY</t>
+          <t>BEN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19.8</v>
+        <v>2021</v>
       </c>
       <c r="C7" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>18.2</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>4.7</v>
+        <v>11.29</v>
       </c>
       <c r="F7" t="n">
-        <v>51.8</v>
+        <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="H7" t="n">
-        <v>67.7</v>
+        <v>606400220.78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>BFA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11.6</v>
+        <v>2021</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>10.7</v>
+        <v>4.38</v>
       </c>
       <c r="E8" t="n">
-        <v>28.9</v>
+        <v>7.82</v>
       </c>
       <c r="F8" t="n">
-        <v>40.7</v>
+        <v>12.73</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
-      </c>
-      <c r="H8" t="n">
-        <v>61.1</v>
+        <v>1226339315.57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KEN</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45.3</v>
+        <v>2021</v>
       </c>
       <c r="C9" t="n">
-        <v>11.3</v>
+        <v>0.31</v>
       </c>
       <c r="D9" t="n">
-        <v>5.2</v>
+        <v>7.96</v>
       </c>
       <c r="E9" t="n">
-        <v>4.8</v>
+        <v>1.15</v>
       </c>
       <c r="F9" t="n">
-        <v>32.9</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>47.9</v>
+        <v>5225078128.78</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CIV</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44.3</v>
-      </c>
-      <c r="C10" t="n">
-        <v>12.4</v>
+        <v>2022</v>
       </c>
       <c r="D10" t="n">
-        <v>15.8</v>
+        <v>14.08</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9</v>
+        <v>15.42</v>
       </c>
       <c r="F10" t="n">
-        <v>13.8</v>
+        <v>14.08</v>
       </c>
       <c r="G10" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="H10" t="n">
-        <v>48.2</v>
+        <v>22459046.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZA</t>
+          <t>CIV</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32.6</v>
+        <v>2021</v>
       </c>
       <c r="C11" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>3.9</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>4.9</v>
+        <v>8.73</v>
       </c>
       <c r="F11" t="n">
-        <v>13.4</v>
+        <v>6.08</v>
       </c>
       <c r="G11" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="H11" t="n">
-        <v>32.7</v>
+        <v>2684932850.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>CMR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>80.3</v>
-      </c>
-      <c r="C12" t="n">
-        <v>9.6</v>
+        <v>2022</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>13.61</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7</v>
+        <v>17.33</v>
       </c>
       <c r="F12" t="n">
-        <v>9.199999999999999</v>
+        <v>13.61</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>19.2</v>
+        <v>371674071.87</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GHA</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>2020</v>
       </c>
       <c r="C13" t="n">
-        <v>1.1</v>
+        <v>9.1</v>
       </c>
       <c r="D13" t="n">
-        <v>24</v>
+        <v>11.46</v>
       </c>
       <c r="E13" t="n">
-        <v>3.7</v>
+        <v>8.32</v>
       </c>
       <c r="F13" t="n">
-        <v>7.8</v>
+        <v>9.23</v>
       </c>
       <c r="G13" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="H13" t="n">
-        <v>39.6</v>
+        <v>1379316852.59</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AGO</t>
+          <t>COG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
+        <v>2022</v>
       </c>
       <c r="D14" t="n">
-        <v>88.90000000000001</v>
+        <v>16.18</v>
       </c>
       <c r="E14" t="n">
-        <v>4.1</v>
+        <v>18.1</v>
       </c>
       <c r="F14" t="n">
-        <v>6.6</v>
+        <v>16.18</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H14" t="n">
-        <v>30.7</v>
+        <v>202024283.93</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="G15" t="n">
+        <v>22904623.97</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E16" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="G16" t="n">
+        <v>35981705.72</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EGY</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F17" t="n">
+        <v>19.22</v>
+      </c>
+      <c r="G17" t="n">
+        <v>761727452.4299999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C18" t="n">
+        <v>13.39</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="E18" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="F18" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1029169935.49</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GAB</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" t="n">
+        <v>17.16</v>
+      </c>
+      <c r="E19" t="n">
+        <v>16.03</v>
+      </c>
+      <c r="F19" t="n">
+        <v>17.16</v>
+      </c>
+      <c r="G19" t="n">
+        <v>186213242.18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GHA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F20" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1570813372.57</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GMB</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="G21" t="n">
+        <v>217160662.91</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="D22" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2082304715.01</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LBR</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="E23" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F23" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="G23" t="n">
+        <v>33434518.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LSO</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1283905541.77</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F25" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2209677095.37</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MDG</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="D26" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F26" t="n">
+        <v>12.33</v>
+      </c>
+      <c r="G26" t="n">
+        <v>674841386.13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MLI</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="F27" t="n">
+        <v>15.46</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2096499380.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MOZ</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2684781614.41</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MRT</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D29" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="F29" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="G29" t="n">
+        <v>439429615.63</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MUS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G30" t="n">
+        <v>626086169.5700001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MWI</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="D31" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="E31" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="G31" t="n">
+        <v>900781299.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NAM</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D32" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12.33</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3108338702.96</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NER</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="F33" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="G33" t="n">
+        <v>613708212.34</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>NGA</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D15" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H15" t="n">
-        <v>29.7</v>
+      <c r="B34" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="E34" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1004758955.42</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D35" t="n">
+        <v>28.71</v>
+      </c>
+      <c r="E35" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="F35" t="n">
+        <v>22.88</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1150118515.52</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SEN</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="E36" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F36" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1303126876.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C37" t="n">
+        <v>20</v>
+      </c>
+      <c r="D37" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="E37" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F37" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="G37" t="n">
+        <v>989374.77</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SWZ</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D38" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F38" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1603658639.66</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SYC</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="G39" t="n">
+        <v>402117461.92</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TGO</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="E40" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="G40" t="n">
+        <v>414699470.15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TZA</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D41" t="n">
+        <v>19.78</v>
+      </c>
+      <c r="E41" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="F41" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1210013969</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>UGA</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D42" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F42" t="n">
+        <v>24.73</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2473782299.73</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ZAF</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E43" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F43" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="G43" t="n">
+        <v>8571329481.81</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ZMB</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="E44" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F44" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="G44" t="n">
+        <v>3116458590.37</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C45" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="E45" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="F45" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="G45" t="n">
+        <v>4096558244.66</v>
       </c>
     </row>
   </sheetData>
@@ -51709,1068 +52540,393 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Arancel aplicado y de nación más favorecida de los países africanos según el origen de las importaciones (%)</t>
+          <t>Exportaciones de los miembros de la PAFTA a otros miembros, con y sin combustibles (% del total)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WITS (Banco Mundial), tradestats-tariff: AHS-WGHTD-AVRG y MFN-WGHTD-AVRG por socio, ponderados por las importaciones de cada socio (MPRT-TRD-VL); último año disponible entre 2019 y 2022. Comunidad = socio de la misma comunidad con libre comercio (CEDEAO, CEEAC, EAC, COMESA, SADC, UEMOA, CEMAC). Cálculo propio (Code/figuras_afinidad.py).</t>
+          <t>WITS (Banco Mundial), exportaciones declaradas por cada miembro, total y grupo «Fuels» (CUCI 3); solo los miembros que declaran cada año (al menos la mitad). El petróleo que se declara sin destino cuenta en el total pero no en ningún socio. Cálculo propio.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>País</t>
+          <t>Año</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Año</t>
+          <t>Todas las exportaciones (%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Aplicado, comunidad</t>
+          <t>Sin combustibles (%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Aplicado, resto de África</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Aplicado, fuera de África</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>NMF, a África</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Importaciones desde África (USD)</t>
+          <t>Miembros que declaran</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AGO</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1999</v>
       </c>
       <c r="B5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B7" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B10" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B11" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B12" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B13" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B14" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B15" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D16" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D17" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B18" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C18" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B19" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C19" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B20" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B21" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="C21" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B22" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="C22" t="n">
+        <v>20</v>
+      </c>
+      <c r="D22" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B23" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B24" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B25" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="C25" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="D25" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B26" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="C26" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>2021</v>
       </c>
-      <c r="C5" t="n">
-        <v>19.71</v>
-      </c>
-      <c r="D5" t="n">
-        <v>13.39</v>
-      </c>
-      <c r="E5" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="F5" t="n">
-        <v>15.64</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1204584255.78</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BDI</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>15.96</v>
-      </c>
-      <c r="E6" t="n">
-        <v>9.17</v>
-      </c>
-      <c r="F6" t="n">
-        <v>24.36</v>
-      </c>
-      <c r="G6" t="n">
-        <v>308315205.21</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BEN</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" t="n">
-        <v>11.29</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="B27" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C27" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="D27" t="n">
         <v>12</v>
       </c>
-      <c r="G7" t="n">
-        <v>606400220.78</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>BFA</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="E8" t="n">
-        <v>7.82</v>
-      </c>
-      <c r="F8" t="n">
-        <v>12.73</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1226339315.57</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>BWA</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="D9" t="n">
-        <v>7.96</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="F9" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="G9" t="n">
-        <v>5225078128.78</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CAF</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
         <v>2022</v>
       </c>
-      <c r="D10" t="n">
-        <v>14.08</v>
-      </c>
-      <c r="E10" t="n">
-        <v>15.42</v>
-      </c>
-      <c r="F10" t="n">
-        <v>14.08</v>
-      </c>
-      <c r="G10" t="n">
-        <v>22459046.35</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CIV</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="E11" t="n">
-        <v>8.73</v>
-      </c>
-      <c r="F11" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2684932850.6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CMR</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D12" t="n">
-        <v>13.61</v>
-      </c>
-      <c r="E12" t="n">
-        <v>17.33</v>
-      </c>
-      <c r="F12" t="n">
-        <v>13.61</v>
-      </c>
-      <c r="G12" t="n">
-        <v>371674071.87</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C13" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="D13" t="n">
-        <v>11.46</v>
-      </c>
-      <c r="E13" t="n">
-        <v>8.32</v>
-      </c>
-      <c r="F13" t="n">
-        <v>9.23</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1379316852.59</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>COG</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D14" t="n">
-        <v>16.18</v>
-      </c>
-      <c r="E14" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="F14" t="n">
-        <v>16.18</v>
-      </c>
-      <c r="G14" t="n">
-        <v>202024283.93</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>COM</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C15" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="D15" t="n">
-        <v>5.07</v>
-      </c>
-      <c r="E15" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F15" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="G15" t="n">
-        <v>22904623.97</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="D16" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>10.22</v>
-      </c>
-      <c r="F16" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="G16" t="n">
-        <v>35981705.72</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>EGY</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C17" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E17" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="F17" t="n">
-        <v>19.22</v>
-      </c>
-      <c r="G17" t="n">
-        <v>761727452.4299999</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C18" t="n">
-        <v>13.39</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="E18" t="n">
-        <v>12.22</v>
-      </c>
-      <c r="F18" t="n">
-        <v>9.380000000000001</v>
-      </c>
-      <c r="G18" t="n">
-        <v>1029169935.49</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>GAB</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C19" t="n">
-        <v>30</v>
-      </c>
-      <c r="D19" t="n">
-        <v>17.16</v>
-      </c>
-      <c r="E19" t="n">
-        <v>16.03</v>
-      </c>
-      <c r="F19" t="n">
-        <v>17.16</v>
-      </c>
-      <c r="G19" t="n">
-        <v>186213242.18</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>GHA</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>9.609999999999999</v>
-      </c>
-      <c r="E20" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="F20" t="n">
-        <v>11.67</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1570813372.57</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>GMB</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="E21" t="n">
-        <v>13.17</v>
-      </c>
-      <c r="F21" t="n">
-        <v>16.61</v>
-      </c>
-      <c r="G21" t="n">
-        <v>217160662.91</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>KEN</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="D22" t="n">
-        <v>10.35</v>
-      </c>
-      <c r="E22" t="n">
-        <v>9.369999999999999</v>
-      </c>
-      <c r="F22" t="n">
-        <v>28.12</v>
-      </c>
-      <c r="G22" t="n">
-        <v>2082304715.01</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>LBR</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>14.02</v>
-      </c>
-      <c r="E23" t="n">
-        <v>10.32</v>
-      </c>
-      <c r="F23" t="n">
-        <v>14.16</v>
-      </c>
-      <c r="G23" t="n">
-        <v>33434518.2</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>LSO</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="n">
-        <v>87.40000000000001</v>
-      </c>
-      <c r="E24" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="F24" t="n">
-        <v>12.27</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1283905541.77</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="E25" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="F25" t="n">
-        <v>12.64</v>
-      </c>
-      <c r="G25" t="n">
-        <v>2209677095.37</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>MDG</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C26" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="D26" t="n">
-        <v>11.28</v>
-      </c>
-      <c r="E26" t="n">
-        <v>7.12</v>
-      </c>
-      <c r="F26" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="G26" t="n">
-        <v>674841386.13</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>MLI</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>10.47</v>
-      </c>
-      <c r="E27" t="n">
-        <v>7.47</v>
-      </c>
-      <c r="F27" t="n">
-        <v>15.46</v>
-      </c>
-      <c r="G27" t="n">
-        <v>2096499380.4</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>MOZ</t>
-        </is>
-      </c>
       <c r="B28" t="n">
-        <v>2021</v>
+        <v>12.9</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>32.3</v>
       </c>
       <c r="D28" t="n">
-        <v>6.61</v>
-      </c>
-      <c r="E28" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F28" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2684781614.41</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>MRT</t>
-        </is>
+      <c r="A29" t="n">
+        <v>2023</v>
       </c>
       <c r="B29" t="n">
-        <v>2021</v>
+        <v>14.5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>32.6</v>
       </c>
       <c r="D29" t="n">
-        <v>9.779999999999999</v>
-      </c>
-      <c r="E29" t="n">
-        <v>8.380000000000001</v>
-      </c>
-      <c r="F29" t="n">
-        <v>9.779999999999999</v>
-      </c>
-      <c r="G29" t="n">
-        <v>439429615.63</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>MUS</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="G30" t="n">
-        <v>626086169.5700001</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>MWI</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C31" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="D31" t="n">
-        <v>9.67</v>
-      </c>
-      <c r="E31" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="F31" t="n">
-        <v>13.12</v>
-      </c>
-      <c r="G31" t="n">
-        <v>900781299.25</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>NAM</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="D32" t="n">
-        <v>14.48</v>
-      </c>
-      <c r="E32" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="F32" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="G32" t="n">
-        <v>3108338702.96</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>NER</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="E33" t="n">
-        <v>9.01</v>
-      </c>
-      <c r="F33" t="n">
-        <v>16.77</v>
-      </c>
-      <c r="G33" t="n">
-        <v>613708212.34</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>NGA</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" t="n">
-        <v>9.08</v>
-      </c>
-      <c r="E34" t="n">
-        <v>10.83</v>
-      </c>
-      <c r="F34" t="n">
-        <v>9.94</v>
-      </c>
-      <c r="G34" t="n">
-        <v>1004758955.42</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>RWA</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="D35" t="n">
-        <v>28.71</v>
-      </c>
-      <c r="E35" t="n">
-        <v>13.62</v>
-      </c>
-      <c r="F35" t="n">
-        <v>22.88</v>
-      </c>
-      <c r="G35" t="n">
-        <v>1150118515.52</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SEN</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>10.87</v>
-      </c>
-      <c r="E36" t="n">
-        <v>9.359999999999999</v>
-      </c>
-      <c r="F36" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="G36" t="n">
-        <v>1303126876.8</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>STP</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C37" t="n">
-        <v>20</v>
-      </c>
-      <c r="D37" t="n">
-        <v>8.210000000000001</v>
-      </c>
-      <c r="E37" t="n">
-        <v>10.87</v>
-      </c>
-      <c r="F37" t="n">
-        <v>9.41</v>
-      </c>
-      <c r="G37" t="n">
-        <v>989374.77</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>SWZ</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D38" t="n">
-        <v>4.87</v>
-      </c>
-      <c r="E38" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="F38" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="G38" t="n">
-        <v>1603658639.66</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>SYC</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="D39" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="E39" t="n">
-        <v>3.65</v>
-      </c>
-      <c r="F39" t="n">
-        <v>3.98</v>
-      </c>
-      <c r="G39" t="n">
-        <v>402117461.92</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>TGO</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" t="n">
-        <v>9.76</v>
-      </c>
-      <c r="E40" t="n">
-        <v>11.27</v>
-      </c>
-      <c r="F40" t="n">
-        <v>12.48</v>
-      </c>
-      <c r="G40" t="n">
-        <v>414699470.15</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>TZA</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="D41" t="n">
-        <v>19.78</v>
-      </c>
-      <c r="E41" t="n">
-        <v>9.630000000000001</v>
-      </c>
-      <c r="F41" t="n">
-        <v>17.23</v>
-      </c>
-      <c r="G41" t="n">
-        <v>1210013969</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>UGA</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="D42" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="E42" t="n">
-        <v>9.52</v>
-      </c>
-      <c r="F42" t="n">
-        <v>24.73</v>
-      </c>
-      <c r="G42" t="n">
-        <v>2473782299.73</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ZAF</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D43" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="E43" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="F43" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="G43" t="n">
-        <v>8571329481.81</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ZMB</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="D44" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="E44" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="F44" t="n">
-        <v>10.31</v>
-      </c>
-      <c r="G44" t="n">
-        <v>3116458590.37</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ZWE</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C45" t="n">
-        <v>11.85</v>
-      </c>
-      <c r="D45" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="E45" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="F45" t="n">
-        <v>11.84</v>
-      </c>
-      <c r="G45" t="n">
-        <v>4096558244.66</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -52784,20 +52940,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Exportaciones de los miembros de la PAFTA a otros miembros, con y sin combustibles (% del total)</t>
+          <t>Composición de las exportaciones de los miembros de la PAFTA a otros miembros y fuera de la PAFTA (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WITS (Banco Mundial), exportaciones declaradas por cada miembro, total y grupo «Fuels» (CUCI 3); solo los miembros que declaran cada año (al menos la mitad). El petróleo que se declara sin destino cuenta en el total pero no en ningún socio. Cálculo propio.</t>
+          <t>WITS (Banco Mundial), exportaciones declaradas por grupos de la CUCI. «Otros y sin clasificar» incluye el petróleo declarado sin desglose de producto. Cálculo propio (Code/figuras_afinidad.py).</t>
         </is>
       </c>
     </row>
@@ -52809,368 +52965,150 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Todas las exportaciones (%)</t>
+          <t>Destino</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sin combustibles (%)</t>
+          <t>Alimentos (%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Miembros que declaran</t>
+          <t>Materias primas agrícolas (%)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Combustibles (%)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Minerales y metales (%)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Manufacturas (%)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Otros (%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1999</v>
-      </c>
-      <c r="B5" t="n">
-        <v>4.5</v>
+        <v>2005</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dentro</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>15.1</v>
+        <v>15.4</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>0.7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>5.4</v>
+        <v>2005</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>23.4</v>
+        <v>1.4</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>0.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2001</v>
-      </c>
-      <c r="B7" t="n">
-        <v>7.7</v>
+        <v>2023</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dentro</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>29.9</v>
+        <v>12.6</v>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>0.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2002</v>
-      </c>
-      <c r="B8" t="n">
-        <v>9</v>
+        <v>2023</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>26.6</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B9" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="C9" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="D9" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2004</v>
-      </c>
-      <c r="B10" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="C10" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="D10" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B11" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="C11" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="D11" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2006</v>
-      </c>
-      <c r="B12" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="C12" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="D12" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>2007</v>
-      </c>
-      <c r="B13" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="C13" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="D13" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B14" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="C14" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="D14" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2009</v>
-      </c>
-      <c r="B15" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="C15" t="n">
-        <v>27</v>
-      </c>
-      <c r="D15" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B16" t="n">
-        <v>9</v>
-      </c>
-      <c r="C16" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="D16" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B17" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="C17" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="D17" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B18" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="C18" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="D18" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B19" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="C19" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="D19" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B20" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G8" t="n">
         <v>21.5</v>
       </c>
-      <c r="D20" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B21" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="C21" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="D21" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B22" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="C22" t="n">
-        <v>20</v>
-      </c>
-      <c r="D22" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B23" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="C23" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="D23" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B24" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="C24" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="D24" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B25" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="C25" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="D25" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B26" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="C26" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="D26" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B27" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="C27" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="D27" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B28" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="C28" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="D28" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B29" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="C29" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="D29" t="n">
-        <v>12</v>
+      <c r="H8" t="n">
+        <v>6.1</v>
       </c>
     </row>
   </sheetData>
@@ -53184,20 +53122,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Composición de las exportaciones de los miembros de la PAFTA a otros miembros y fuera de la PAFTA (%)</t>
+          <t>Manufacturas en las exportaciones de los países africanos a África y fuera de África (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WITS (Banco Mundial), exportaciones declaradas por grupos de la CUCI. «Otros y sin clasificar» incluye el petróleo declarado sin desglose de producto. Cálculo propio (Code/figuras_afinidad.py).</t>
+          <t>WITS (Banco Mundial), grupo «manuf» (CUCI 5 a 8 sin 667 y 68) y total, exportaciones declaradas por cada país a cada socio; solo los países que declaran cada año. Cálculo propio (Code/figuras_afinidad.py).</t>
         </is>
       </c>
     </row>
@@ -53209,150 +53147,212 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Destino</t>
+          <t>A África (%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Alimentos (%)</t>
+          <t>Fuera de África (%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Materias primas agrícolas (%)</t>
+          <t>Países que declaran</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Combustibles (%)</t>
+          <t>AGO 2023: África / fuera</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Minerales y metales (%)</t>
+          <t>TUN 2023: África / fuera</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Manufacturas (%)</t>
+          <t>MAR 2023: África / fuera</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Otros (%)</t>
+          <t>EGY 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ZAF 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>KEN 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>GHA 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CIV 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>TZA 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ETH 2023: África / fuera</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>NGA 2023: África / fuera</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Dentro</t>
-        </is>
+        <v>2000</v>
+      </c>
+      <c r="B5" t="n">
+        <v>40.6</v>
       </c>
       <c r="C5" t="n">
-        <v>15.4</v>
+        <v>26.2</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>8.300000000000001</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>2005</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fuera</t>
-        </is>
+      <c r="B6" t="n">
+        <v>45.3</v>
       </c>
       <c r="C6" t="n">
-        <v>1.4</v>
+        <v>27.2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>76.7</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>9.4</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Dentro</t>
-        </is>
+        <v>2010</v>
+      </c>
+      <c r="B7" t="n">
+        <v>45.7</v>
       </c>
       <c r="C7" t="n">
-        <v>12.6</v>
+        <v>20.6</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E7" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="H7" t="n">
-        <v>6.7</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B8" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B9" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
         <v>2023</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Fuera</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>67.3</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G8" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>6.1</v>
+      <c r="B10" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>72.8 / 2.4</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>71.9 / 80.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>70.9 / 75.2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>69.0 / 48.2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>61.9 / 32.9</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>57.6 / 14.3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>33.3 / 1.2</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>32.7 / 6.8</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>27.4 / 5.3</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>13.9 / 8.4</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>8.5 / 2.2</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>